<commit_message>
Treat Palconn DDP as net warehouse cost; score vs Gator.
Rings lose money at Gator/site. Sticks and PPSU workhorses make ~25–38% GM, not 50%.

Co-authored-by: baruchstablet <baruchstablet@gmail.com>
</commit_message>
<xml_diff>
--- a/cursor/product-pricing-analysis/palconn/Palconn_15Sep_DDP_vs_landed.xlsx
+++ b/cursor/product-pricing-analysis/palconn/Palconn_15Sep_DDP_vs_landed.xlsx
@@ -4304,21 +4304,21 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>True DDP to the warehouse should also cover entry, DTHC, chassis, and dray to Livingston.</t>
+          <t>True DDP to the warehouse: Baruch confirmed 16 Sep her DDP includes delivery to Livingston — no dest add-on.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Palconn DDP sitting ~1% under FOB×1.43+ocean (which already excludes those dest fees) means this is</t>
+          <t>Palconn DDP sitting ~1% under FOB×1.43+ocean means the formula already approximates all-in warehouse cost.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>duty+ocean math, not proven door-to-door. Prefer FOB + our forwarder on the first buy.</t>
+          <t>Sell cards = Gator/NJPD (quote 11237145, ack 11234952), rounded up on the site. Rings lose money at Gator; sticks/PPSU ~25–38% GM.</t>
         </is>
       </c>
     </row>

</xml_diff>